<commit_message>
feat: Add Area column to table_license and area filter checkboxes in Dashboard
- Backend: Add area TEXT column to table_license schema
- Backend: Safe ALTER TABLE migration (no data loss on existing DB)
- Backend: Default area values: GGPD->KV1, GGHL0->KV2, GGHL1->KV3
- Backend: Update SQL hint in table_schedules for license table
- Frontend: Add Area to TABLE_TEMPLATES.license (columns, sqlHint, rows)
- Frontend: Column D now reads area from licMatch instead of hardcoded KV1
- Frontend: Add Area field to generateClientMockData license objects
- Frontend: Add selectedAreas state and allAreas memo derived from column D
- Frontend: filteredDashRows now filters by area AND node simultaneously
- Frontend: Add Area filter checkbox bar (violet theme) in Dashboard tab
  - Shows each distinct area with node count
  - Toggle checkbox to filter charts by area
  - Clear button to reset area filter
</commit_message>
<xml_diff>
--- a/input/GGSN_lic.xlsx
+++ b/input/GGSN_lic.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\longvh3\Downloads\Tinh_tai_UCTT\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BBF3F2F-C317-4DB9-A6BC-36D2C6D7F2D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48F2A0E5-3AD4-4D8B-9D50-7C4ED7018211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{86FB7837-5156-4E66-8194-3534D6D55526}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="82">
   <si>
     <t>Node</t>
   </si>
@@ -268,6 +268,18 @@
   </si>
   <si>
     <t>GGHT24</t>
+  </si>
+  <si>
+    <t>Area</t>
+  </si>
+  <si>
+    <t>KV1</t>
+  </si>
+  <si>
+    <t>KV2</t>
+  </si>
+  <si>
+    <t>KV3</t>
   </si>
 </sst>
 </file>
@@ -734,1392 +746,1599 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23258FE4-BBCC-4ACD-9ED6-A704A2594A9B}">
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="10.140625" customWidth="1"/>
-    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="3" width="10.140625" customWidth="1"/>
+    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="22.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="C2">
-        <v>4500000</v>
+      <c r="C2" s="9" t="s">
+        <v>79</v>
       </c>
       <c r="D2">
-        <v>150000</v>
+        <v>4500000</v>
       </c>
       <c r="E2">
-        <v>4500000</v>
+        <v>150000</v>
       </c>
       <c r="F2">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4500000</v>
+      </c>
+      <c r="G2">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="C3">
-        <v>4500000</v>
+      <c r="C3" s="9" t="s">
+        <v>79</v>
       </c>
       <c r="D3">
-        <v>150000</v>
+        <v>4500000</v>
       </c>
       <c r="E3">
-        <v>4500000</v>
+        <v>150000</v>
       </c>
       <c r="F3">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4500000</v>
+      </c>
+      <c r="G3">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D4">
         <v>3500000</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>100000</v>
       </c>
-      <c r="E4">
-        <v>4500000</v>
-      </c>
       <c r="F4">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4500000</v>
+      </c>
+      <c r="G4">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="C5">
-        <v>4500000</v>
+      <c r="C5" s="9" t="s">
+        <v>79</v>
       </c>
       <c r="D5">
-        <v>150000</v>
+        <v>4500000</v>
       </c>
       <c r="E5">
-        <v>4500000</v>
+        <v>150000</v>
       </c>
       <c r="F5">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4500000</v>
+      </c>
+      <c r="G5">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6">
         <v>1500000</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>60000</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>1500000</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>80000</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D7">
         <v>1500000</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <v>60000</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <v>1500000</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <v>80000</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D8">
         <v>1500000</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>60000</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <v>1500000</v>
       </c>
-      <c r="F8">
+      <c r="G8">
         <v>80000</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D9">
         <v>1500000</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <v>60000</v>
       </c>
-      <c r="E9">
+      <c r="F9">
         <v>1500000</v>
       </c>
-      <c r="F9">
+      <c r="G9">
         <v>80000</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D10">
         <v>2800000</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>135000</v>
       </c>
-      <c r="E10">
+      <c r="F10">
         <v>2800000</v>
       </c>
-      <c r="F10">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D11">
         <v>2800000</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>135000</v>
       </c>
-      <c r="E11">
+      <c r="F11">
         <v>2800000</v>
       </c>
-      <c r="F11">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D12">
         <v>2800000</v>
       </c>
-      <c r="D12">
+      <c r="E12">
         <v>135000</v>
       </c>
-      <c r="E12">
+      <c r="F12">
         <v>2800000</v>
       </c>
-      <c r="F12">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D13">
         <v>2800000</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <v>135000</v>
       </c>
-      <c r="E13">
+      <c r="F13">
         <v>2800000</v>
       </c>
-      <c r="F13">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D14">
         <v>2900000</v>
       </c>
-      <c r="D14">
+      <c r="E14">
         <v>100000</v>
       </c>
-      <c r="E14">
+      <c r="F14">
         <v>2400000</v>
       </c>
-      <c r="F14">
+      <c r="G14">
         <v>100000</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>18</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="C15">
-        <v>4000000</v>
+      <c r="C15" s="9" t="s">
+        <v>79</v>
       </c>
       <c r="D15">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E15">
-        <v>4000000</v>
+        <v>150000</v>
       </c>
       <c r="F15">
+        <v>4000000</v>
+      </c>
+      <c r="G15">
         <v>180000</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>19</v>
       </c>
       <c r="B16" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="C16">
-        <v>0</v>
+      <c r="C16" s="9" t="s">
+        <v>79</v>
       </c>
       <c r="D16">
         <v>0</v>
       </c>
       <c r="E16">
-        <v>4000000</v>
+        <v>0</v>
       </c>
       <c r="F16">
+        <v>4000000</v>
+      </c>
+      <c r="G16">
         <v>180000</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>20</v>
       </c>
       <c r="B17" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="C17">
-        <v>4000000</v>
+      <c r="C17" s="9" t="s">
+        <v>79</v>
       </c>
       <c r="D17">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E17">
-        <v>4000000</v>
+        <v>150000</v>
       </c>
       <c r="F17">
+        <v>4000000</v>
+      </c>
+      <c r="G17">
         <v>180000</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>21</v>
       </c>
       <c r="B18" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="C18">
-        <v>4000000</v>
+      <c r="C18" s="9" t="s">
+        <v>79</v>
       </c>
       <c r="D18">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E18">
-        <v>4000000</v>
+        <v>150000</v>
       </c>
       <c r="F18">
+        <v>4000000</v>
+      </c>
+      <c r="G18">
         <v>180000</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
       <c r="B19" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="C19">
-        <v>4000000</v>
+      <c r="C19" s="9" t="s">
+        <v>79</v>
       </c>
       <c r="D19">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E19">
-        <v>4000000</v>
+        <v>150000</v>
       </c>
       <c r="F19">
+        <v>4000000</v>
+      </c>
+      <c r="G19">
         <v>180000</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>23</v>
       </c>
       <c r="B20" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="C20">
-        <v>0</v>
+      <c r="C20" s="9" t="s">
+        <v>79</v>
       </c>
       <c r="D20">
         <v>0</v>
       </c>
       <c r="E20">
-        <v>4000000</v>
+        <v>0</v>
       </c>
       <c r="F20">
+        <v>4000000</v>
+      </c>
+      <c r="G20">
         <v>180000</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="C21">
-        <v>0</v>
+      <c r="C21" s="9" t="s">
+        <v>79</v>
       </c>
       <c r="D21">
         <v>0</v>
       </c>
       <c r="E21">
-        <v>4000000</v>
+        <v>0</v>
       </c>
       <c r="F21">
+        <v>4000000</v>
+      </c>
+      <c r="G21">
         <v>180000</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>25</v>
       </c>
       <c r="B22" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="C22">
-        <v>0</v>
+      <c r="C22" s="9" t="s">
+        <v>79</v>
       </c>
       <c r="D22">
         <v>0</v>
       </c>
       <c r="E22">
-        <v>4000000</v>
+        <v>0</v>
       </c>
       <c r="F22">
+        <v>4000000</v>
+      </c>
+      <c r="G22">
         <v>180000</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>26</v>
       </c>
       <c r="B23" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D23">
         <v>3500000</v>
       </c>
-      <c r="D23">
+      <c r="E23">
         <v>100000</v>
       </c>
-      <c r="E23">
+      <c r="F23">
         <v>3500000</v>
       </c>
-      <c r="F23">
+      <c r="G23">
         <v>100000</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>27</v>
       </c>
       <c r="B24" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="C24">
+      <c r="C24" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D24">
         <v>3500000</v>
       </c>
-      <c r="D24">
+      <c r="E24">
         <v>100000</v>
       </c>
-      <c r="E24">
+      <c r="F24">
         <v>3500000</v>
       </c>
-      <c r="F24">
+      <c r="G24">
         <v>100000</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>28</v>
       </c>
       <c r="B25" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="C25">
-        <v>4500000</v>
+      <c r="C25" s="9" t="s">
+        <v>79</v>
       </c>
       <c r="D25">
-        <v>150000</v>
+        <v>4500000</v>
       </c>
       <c r="E25">
-        <v>4500000</v>
+        <v>150000</v>
       </c>
       <c r="F25">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4500000</v>
+      </c>
+      <c r="G25">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>29</v>
       </c>
       <c r="B26" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="C26">
-        <v>4500000</v>
+      <c r="C26" s="9" t="s">
+        <v>79</v>
       </c>
       <c r="D26">
-        <v>150000</v>
+        <v>4500000</v>
       </c>
       <c r="E26">
-        <v>4500000</v>
+        <v>150000</v>
       </c>
       <c r="F26">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4500000</v>
+      </c>
+      <c r="G26">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>66</v>
       </c>
       <c r="B27" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="C27">
-        <v>4500000</v>
+      <c r="C27" s="9" t="s">
+        <v>79</v>
       </c>
       <c r="D27">
-        <v>150000</v>
+        <v>4500000</v>
       </c>
       <c r="E27">
-        <v>4500000</v>
+        <v>150000</v>
       </c>
       <c r="F27">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4500000</v>
+      </c>
+      <c r="G27">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>67</v>
       </c>
       <c r="B28" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="C28">
-        <v>4500000</v>
+      <c r="C28" s="9" t="s">
+        <v>79</v>
       </c>
       <c r="D28">
-        <v>150000</v>
+        <v>4500000</v>
       </c>
       <c r="E28">
-        <v>4500000</v>
+        <v>150000</v>
       </c>
       <c r="F28">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4500000</v>
+      </c>
+      <c r="G28">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>68</v>
       </c>
       <c r="B29" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="C29">
-        <v>4500000</v>
+      <c r="C29" s="9" t="s">
+        <v>79</v>
       </c>
       <c r="D29">
-        <v>150000</v>
+        <v>4500000</v>
       </c>
       <c r="E29">
-        <v>4500000</v>
+        <v>150000</v>
       </c>
       <c r="F29">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4500000</v>
+      </c>
+      <c r="G29">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>69</v>
       </c>
       <c r="B30" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="C30">
-        <v>4500000</v>
+      <c r="C30" s="9" t="s">
+        <v>79</v>
       </c>
       <c r="D30">
-        <v>150000</v>
+        <v>4500000</v>
       </c>
       <c r="E30">
-        <v>4500000</v>
+        <v>150000</v>
       </c>
       <c r="F30">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4500000</v>
+      </c>
+      <c r="G30">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>30</v>
       </c>
       <c r="B31" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="C31">
+      <c r="C31" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="D31">
         <v>1500000</v>
       </c>
-      <c r="D31">
+      <c r="E31">
         <v>60000</v>
       </c>
-      <c r="E31">
+      <c r="F31">
         <v>1500000</v>
       </c>
-      <c r="F31">
+      <c r="G31">
         <v>80000</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>31</v>
       </c>
       <c r="B32" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="C32">
+      <c r="C32" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="D32">
         <v>1500000</v>
       </c>
-      <c r="D32">
+      <c r="E32">
         <v>60000</v>
       </c>
-      <c r="E32">
+      <c r="F32">
         <v>1500000</v>
       </c>
-      <c r="F32">
+      <c r="G32">
         <v>80000</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>32</v>
       </c>
       <c r="B33" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="C33">
+      <c r="C33" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="D33">
         <v>2000000</v>
       </c>
-      <c r="D33">
+      <c r="E33">
         <v>70000</v>
       </c>
-      <c r="E33">
+      <c r="F33">
         <v>2000000</v>
       </c>
-      <c r="F33">
+      <c r="G33">
         <v>100000</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
         <v>33</v>
       </c>
       <c r="B34" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="C34">
+      <c r="C34" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="D34">
         <v>1800000</v>
       </c>
-      <c r="D34">
+      <c r="E34">
         <v>90000</v>
       </c>
-      <c r="E34">
+      <c r="F34">
         <v>1800000</v>
       </c>
-      <c r="F34">
+      <c r="G34">
         <v>100000</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
         <v>34</v>
       </c>
       <c r="B35" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="C35">
-        <v>4000000</v>
+      <c r="C35" s="12" t="s">
+        <v>80</v>
       </c>
       <c r="D35">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E35">
-        <v>4000000</v>
+        <v>150000</v>
       </c>
       <c r="F35">
+        <v>4000000</v>
+      </c>
+      <c r="G35">
         <v>180000</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="7" t="s">
         <v>35</v>
       </c>
       <c r="B36" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="C36">
-        <v>4000000</v>
+      <c r="C36" s="12" t="s">
+        <v>80</v>
       </c>
       <c r="D36">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E36">
-        <v>4000000</v>
+        <v>150000</v>
       </c>
       <c r="F36">
+        <v>4000000</v>
+      </c>
+      <c r="G36">
         <v>180000</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
         <v>36</v>
       </c>
       <c r="B37" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="C37">
-        <v>4000000</v>
+      <c r="C37" s="12" t="s">
+        <v>80</v>
       </c>
       <c r="D37">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E37">
-        <v>4000000</v>
+        <v>150000</v>
       </c>
       <c r="F37">
+        <v>4000000</v>
+      </c>
+      <c r="G37">
         <v>180000</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="7" t="s">
         <v>37</v>
       </c>
       <c r="B38" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="C38">
-        <v>4000000</v>
+      <c r="C38" s="12" t="s">
+        <v>80</v>
       </c>
       <c r="D38">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E38">
+        <v>150000</v>
+      </c>
+      <c r="F38">
         <v>3000000</v>
       </c>
-      <c r="F38">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G38">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
         <v>38</v>
       </c>
       <c r="B39" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="C39">
-        <v>4000000</v>
+      <c r="C39" s="12" t="s">
+        <v>80</v>
       </c>
       <c r="D39">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E39">
+        <v>150000</v>
+      </c>
+      <c r="F39">
         <v>3000000</v>
       </c>
-      <c r="F39">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G39">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
         <v>39</v>
       </c>
       <c r="B40" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="C40">
-        <v>4000000</v>
+      <c r="C40" s="12" t="s">
+        <v>80</v>
       </c>
       <c r="D40">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E40">
+        <v>150000</v>
+      </c>
+      <c r="F40">
         <v>3000000</v>
       </c>
-      <c r="F40">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G40">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>40</v>
       </c>
       <c r="B41" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="C41">
-        <v>4500000</v>
+      <c r="C41" s="12" t="s">
+        <v>80</v>
       </c>
       <c r="D41">
-        <v>150000</v>
+        <v>4500000</v>
       </c>
       <c r="E41">
+        <v>150000</v>
+      </c>
+      <c r="F41">
         <v>3000000</v>
       </c>
-      <c r="F41">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G41">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
         <v>41</v>
       </c>
       <c r="B42" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="C42">
-        <v>4500000</v>
+      <c r="C42" s="12" t="s">
+        <v>80</v>
       </c>
       <c r="D42">
-        <v>150000</v>
+        <v>4500000</v>
       </c>
       <c r="E42">
+        <v>150000</v>
+      </c>
+      <c r="F42">
         <v>3000000</v>
       </c>
-      <c r="F42">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G42">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>70</v>
       </c>
       <c r="B43" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="C43">
-        <v>4000000</v>
+      <c r="C43" s="12" t="s">
+        <v>80</v>
       </c>
       <c r="D43">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E43">
+        <v>150000</v>
+      </c>
+      <c r="F43">
         <v>3000000</v>
       </c>
-      <c r="F43">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G43">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
         <v>71</v>
       </c>
       <c r="B44" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="C44">
-        <v>4000000</v>
+      <c r="C44" s="12" t="s">
+        <v>80</v>
       </c>
       <c r="D44">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E44">
+        <v>150000</v>
+      </c>
+      <c r="F44">
         <v>3000000</v>
       </c>
-      <c r="F44">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G44">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
         <v>72</v>
       </c>
       <c r="B45" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="C45">
-        <v>4000000</v>
+      <c r="C45" s="12" t="s">
+        <v>80</v>
       </c>
       <c r="D45">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E45">
+        <v>150000</v>
+      </c>
+      <c r="F45">
         <v>3000000</v>
       </c>
-      <c r="F45">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G45">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
         <v>73</v>
       </c>
       <c r="B46" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="C46">
-        <v>4000000</v>
+      <c r="C46" s="12" t="s">
+        <v>80</v>
       </c>
       <c r="D46">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E46">
+        <v>150000</v>
+      </c>
+      <c r="F46">
         <v>3000000</v>
       </c>
-      <c r="F46">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G46">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
         <v>74</v>
       </c>
       <c r="B47" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="C47">
-        <v>4000000</v>
+      <c r="C47" s="12" t="s">
+        <v>80</v>
       </c>
       <c r="D47">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E47">
+        <v>150000</v>
+      </c>
+      <c r="F47">
         <v>3000000</v>
       </c>
-      <c r="F47">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G47">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
         <v>42</v>
       </c>
       <c r="B48" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="C48">
+      <c r="C48" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="D48">
         <v>1500000</v>
       </c>
-      <c r="D48">
+      <c r="E48">
         <v>60000</v>
       </c>
-      <c r="E48">
+      <c r="F48">
         <v>1500000</v>
       </c>
-      <c r="F48">
+      <c r="G48">
         <v>80000</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
         <v>43</v>
       </c>
       <c r="B49" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="C49">
+      <c r="C49" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="D49">
         <v>1500000</v>
       </c>
-      <c r="D49">
+      <c r="E49">
         <v>60000</v>
       </c>
-      <c r="E49">
+      <c r="F49">
         <v>1500000</v>
       </c>
-      <c r="F49">
+      <c r="G49">
         <v>80000</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>44</v>
       </c>
       <c r="B50" t="s">
         <v>63</v>
       </c>
-      <c r="C50">
+      <c r="C50" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="D50">
         <v>1500000</v>
       </c>
-      <c r="D50">
+      <c r="E50">
         <v>60000</v>
       </c>
-      <c r="E50">
+      <c r="F50">
         <v>1500000</v>
       </c>
-      <c r="F50">
+      <c r="G50">
         <v>80000</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
         <v>45</v>
       </c>
       <c r="B51" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C51">
+      <c r="C51" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="D51">
         <v>2700000</v>
       </c>
-      <c r="D51">
+      <c r="E51">
         <v>130000</v>
       </c>
-      <c r="E51">
+      <c r="F51">
         <v>2700000</v>
       </c>
-      <c r="F51">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G51">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
         <v>46</v>
       </c>
       <c r="B52" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C52">
+      <c r="C52" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="D52">
         <v>1500000</v>
       </c>
-      <c r="D52">
+      <c r="E52">
         <v>60000</v>
       </c>
-      <c r="E52">
+      <c r="F52">
         <v>1500000</v>
       </c>
-      <c r="F52">
+      <c r="G52">
         <v>80000</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
         <v>47</v>
       </c>
       <c r="B53" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C53">
+      <c r="C53" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="D53">
         <v>2500000</v>
       </c>
-      <c r="D53">
+      <c r="E53">
         <v>120000</v>
       </c>
-      <c r="E53">
+      <c r="F53">
         <v>2500000</v>
       </c>
-      <c r="F53">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G53">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="8" t="s">
         <v>48</v>
       </c>
       <c r="B54" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="C54">
+      <c r="C54" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="D54">
         <v>2700000</v>
       </c>
-      <c r="D54">
+      <c r="E54">
         <v>130000</v>
       </c>
-      <c r="E54">
+      <c r="F54">
         <v>2700000</v>
       </c>
-      <c r="F54">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G54">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
         <v>49</v>
       </c>
       <c r="B55" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="C55">
-        <v>4000000</v>
+      <c r="C55" s="11" t="s">
+        <v>81</v>
       </c>
       <c r="D55">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E55">
-        <v>4500000</v>
+        <v>150000</v>
       </c>
       <c r="F55">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4500000</v>
+      </c>
+      <c r="G55">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="8" t="s">
         <v>50</v>
       </c>
       <c r="B56" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="C56">
-        <v>4000000</v>
+      <c r="C56" s="11" t="s">
+        <v>81</v>
       </c>
       <c r="D56">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E56">
-        <v>4500000</v>
+        <v>150000</v>
       </c>
       <c r="F56">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4500000</v>
+      </c>
+      <c r="G56">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
         <v>51</v>
       </c>
       <c r="B57" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="C57">
-        <v>4000000</v>
+      <c r="C57" s="11" t="s">
+        <v>81</v>
       </c>
       <c r="D57">
+        <v>4000000</v>
+      </c>
+      <c r="E57">
         <v>100000</v>
       </c>
-      <c r="E57">
-        <v>4500000</v>
-      </c>
       <c r="F57">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4500000</v>
+      </c>
+      <c r="G57">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>52</v>
       </c>
       <c r="B58" t="s">
         <v>62</v>
       </c>
-      <c r="C58">
-        <v>4000000</v>
+      <c r="C58" s="11" t="s">
+        <v>81</v>
       </c>
       <c r="D58">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E58">
-        <v>4500000</v>
+        <v>150000</v>
       </c>
       <c r="F58">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4500000</v>
+      </c>
+      <c r="G58">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>53</v>
       </c>
       <c r="B59" t="s">
         <v>64</v>
       </c>
-      <c r="C59">
-        <v>4500000</v>
+      <c r="C59" s="11" t="s">
+        <v>81</v>
       </c>
       <c r="D59">
-        <v>150000</v>
+        <v>4500000</v>
       </c>
       <c r="E59">
-        <v>4500000</v>
+        <v>150000</v>
       </c>
       <c r="F59">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4500000</v>
+      </c>
+      <c r="G59">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>54</v>
       </c>
       <c r="B60" t="s">
         <v>64</v>
       </c>
-      <c r="C60">
-        <v>4500000</v>
+      <c r="C60" s="11" t="s">
+        <v>81</v>
       </c>
       <c r="D60">
-        <v>150000</v>
+        <v>4500000</v>
       </c>
       <c r="E60">
-        <v>4500000</v>
+        <v>150000</v>
       </c>
       <c r="F60">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4500000</v>
+      </c>
+      <c r="G60">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>55</v>
       </c>
       <c r="B61" t="s">
         <v>64</v>
       </c>
-      <c r="C61">
-        <v>4500000</v>
+      <c r="C61" s="11" t="s">
+        <v>81</v>
       </c>
       <c r="D61">
-        <v>150000</v>
+        <v>4500000</v>
       </c>
       <c r="E61">
-        <v>4500000</v>
+        <v>150000</v>
       </c>
       <c r="F61">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4500000</v>
+      </c>
+      <c r="G61">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>56</v>
       </c>
       <c r="B62" t="s">
         <v>64</v>
       </c>
-      <c r="C62">
-        <v>4000000</v>
+      <c r="C62" s="11" t="s">
+        <v>81</v>
       </c>
       <c r="D62">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E62">
-        <v>4000000</v>
+        <v>150000</v>
       </c>
       <c r="F62">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4000000</v>
+      </c>
+      <c r="G62">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>57</v>
       </c>
       <c r="B63" t="s">
         <v>65</v>
       </c>
-      <c r="C63">
-        <v>0</v>
+      <c r="C63" s="11" t="s">
+        <v>81</v>
       </c>
       <c r="D63">
         <v>0</v>
       </c>
       <c r="E63">
+        <v>0</v>
+      </c>
+      <c r="F63">
         <v>1700000</v>
       </c>
-      <c r="F63">
+      <c r="G63">
         <v>100000</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>58</v>
       </c>
       <c r="B64" t="s">
         <v>65</v>
       </c>
-      <c r="C64">
-        <v>0</v>
+      <c r="C64" s="11" t="s">
+        <v>81</v>
       </c>
       <c r="D64">
         <v>0</v>
       </c>
       <c r="E64">
+        <v>0</v>
+      </c>
+      <c r="F64">
         <v>1700000</v>
       </c>
-      <c r="F64">
+      <c r="G64">
         <v>100000</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>59</v>
       </c>
       <c r="B65" t="s">
         <v>65</v>
       </c>
-      <c r="C65">
-        <v>0</v>
+      <c r="C65" s="11" t="s">
+        <v>81</v>
       </c>
       <c r="D65">
         <v>0</v>
       </c>
       <c r="E65">
+        <v>0</v>
+      </c>
+      <c r="F65">
         <v>1700000</v>
       </c>
-      <c r="F65">
+      <c r="G65">
         <v>100000</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>60</v>
       </c>
       <c r="B66" t="s">
         <v>65</v>
       </c>
-      <c r="C66">
-        <v>0</v>
+      <c r="C66" s="11" t="s">
+        <v>81</v>
       </c>
       <c r="D66">
         <v>0</v>
       </c>
       <c r="E66">
+        <v>0</v>
+      </c>
+      <c r="F66">
         <v>1700000</v>
       </c>
-      <c r="F66">
+      <c r="G66">
         <v>100000</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>75</v>
       </c>
       <c r="B67" t="s">
         <v>62</v>
       </c>
-      <c r="C67">
-        <v>4000000</v>
+      <c r="C67" s="11" t="s">
+        <v>81</v>
       </c>
       <c r="D67">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E67">
+        <v>150000</v>
+      </c>
+      <c r="F67">
         <v>3500000</v>
       </c>
-      <c r="F67">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G67">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>76</v>
       </c>
       <c r="B68" t="s">
         <v>62</v>
       </c>
-      <c r="C68">
-        <v>4000000</v>
+      <c r="C68" s="11" t="s">
+        <v>81</v>
       </c>
       <c r="D68">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E68">
+        <v>150000</v>
+      </c>
+      <c r="F68">
         <v>3500000</v>
       </c>
-      <c r="F68">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G68">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>77</v>
       </c>
       <c r="B69" t="s">
         <v>62</v>
       </c>
-      <c r="C69">
-        <v>4000000</v>
+      <c r="C69" s="11" t="s">
+        <v>81</v>
       </c>
       <c r="D69">
-        <v>150000</v>
+        <v>4000000</v>
       </c>
       <c r="E69">
+        <v>150000</v>
+      </c>
+      <c r="F69">
         <v>3500000</v>
       </c>
-      <c r="F69">
+      <c r="G69">
         <v>150000</v>
       </c>
     </row>

</xml_diff>